<commit_message>
bugfix: excel missing okay
</commit_message>
<xml_diff>
--- a/week06_codecamp_presentations/codecamp-eval-helper.xlsx
+++ b/week06_codecamp_presentations/codecamp-eval-helper.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://dtudk.sharepoint.com/sites/46120PiWEInternal/Delte dokumenter/General/project_descriptions/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rink\git\G-PiWE\46120-PiWE\week06_codecamp_presentations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="32" documentId="13_ncr:1_{45180FA7-05B4-4035-AC09-35B7C133CD81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{34D4D0E9-92BF-43FE-B2EC-F326CF7D228A}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45A672F8-ED4D-43DC-B81E-A7D1C8AB0E0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ark1" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="31">
   <si>
     <t>Category</t>
   </si>
@@ -121,6 +121,9 @@
   </si>
   <si>
     <t>(insert name)</t>
+  </si>
+  <si>
+    <t>Okay</t>
   </si>
 </sst>
 </file>
@@ -316,7 +319,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -343,19 +346,15 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Heading 3" xfId="1" builtinId="18"/>
@@ -642,31 +641,29 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:T19"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:J49"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.08984375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="45.7265625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="4.81640625" customWidth="1"/>
-    <col min="5" max="5" width="12.7265625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="25.7265625" customWidth="1"/>
-    <col min="7" max="7" width="12.7265625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="25.7265625" customWidth="1"/>
-    <col min="9" max="9" width="12.7265625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="25.7265625" customWidth="1"/>
+    <col min="2" max="2" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="45.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="4.85546875" customWidth="1"/>
+    <col min="5" max="5" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="25.7109375" customWidth="1"/>
+    <col min="7" max="7" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="25.7109375" customWidth="1"/>
+    <col min="9" max="9" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="25.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="19" t="s">
         <v>21</v>
       </c>
       <c r="B1" s="19"/>
       <c r="C1" s="18"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-    </row>
-    <row r="3" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="3" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -677,20 +674,20 @@
         <v>1</v>
       </c>
       <c r="D3" s="1"/>
-      <c r="E3" s="21" t="s">
+      <c r="E3" s="23" t="s">
         <v>22</v>
       </c>
-      <c r="F3" s="22"/>
-      <c r="G3" s="21" t="s">
+      <c r="F3" s="24"/>
+      <c r="G3" s="23" t="s">
         <v>23</v>
       </c>
-      <c r="H3" s="22"/>
-      <c r="I3" s="21" t="s">
+      <c r="H3" s="24"/>
+      <c r="I3" s="23" t="s">
         <v>24</v>
       </c>
-      <c r="J3" s="22"/>
-    </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="J3" s="24"/>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E4" s="3" t="s">
         <v>14</v>
       </c>
@@ -709,29 +706,23 @@
       <c r="J4" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="T4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.35">
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E5" s="3"/>
       <c r="F5" s="8"/>
       <c r="G5" s="3"/>
       <c r="H5" s="8"/>
       <c r="I5" s="3"/>
       <c r="J5" s="8"/>
-      <c r="T5" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.35">
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="B6" s="24" t="s">
+      <c r="B6" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="C6" s="23" t="s">
+      <c r="C6" s="4" t="s">
         <v>25</v>
       </c>
       <c r="D6" s="4"/>
@@ -741,13 +732,10 @@
       <c r="H6" s="12"/>
       <c r="I6" s="5"/>
       <c r="J6" s="12"/>
-      <c r="T6" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.35">
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="7"/>
-      <c r="B7" s="25"/>
+      <c r="B7" s="18"/>
       <c r="C7" s="16" t="s">
         <v>4</v>
       </c>
@@ -757,13 +745,10 @@
       <c r="H7" s="13"/>
       <c r="I7" s="3"/>
       <c r="J7" s="13"/>
-      <c r="T7" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.35">
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="9"/>
-      <c r="B8" s="26"/>
+      <c r="B8" s="21"/>
       <c r="C8" s="10" t="s">
         <v>26</v>
       </c>
@@ -774,13 +759,9 @@
       <c r="H8" s="14"/>
       <c r="I8" s="11"/>
       <c r="J8" s="14"/>
-      <c r="T8" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.35">
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="2"/>
-      <c r="B9" s="27"/>
       <c r="E9" s="3"/>
       <c r="F9" s="13"/>
       <c r="G9" s="3"/>
@@ -788,11 +769,11 @@
       <c r="I9" s="3"/>
       <c r="J9" s="13"/>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="B10" s="28"/>
+      <c r="B10" s="22"/>
       <c r="C10" s="15" t="s">
         <v>3</v>
       </c>
@@ -804,9 +785,9 @@
       <c r="I10" s="5"/>
       <c r="J10" s="12"/>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="7"/>
-      <c r="B11" s="25"/>
+      <c r="B11" s="18"/>
       <c r="C11" s="16" t="s">
         <v>6</v>
       </c>
@@ -817,9 +798,9 @@
       <c r="I11" s="3"/>
       <c r="J11" s="13"/>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="7"/>
-      <c r="B12" s="25"/>
+      <c r="B12" s="18"/>
       <c r="C12" s="16" t="s">
         <v>13</v>
       </c>
@@ -830,9 +811,9 @@
       <c r="I12" s="3"/>
       <c r="J12" s="13"/>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="7"/>
-      <c r="B13" s="25"/>
+      <c r="B13" s="18"/>
       <c r="C13" t="s">
         <v>7</v>
       </c>
@@ -843,9 +824,9 @@
       <c r="I13" s="3"/>
       <c r="J13" s="13"/>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="7"/>
-      <c r="B14" s="25"/>
+      <c r="B14" s="18"/>
       <c r="C14" t="s">
         <v>8</v>
       </c>
@@ -856,9 +837,9 @@
       <c r="I14" s="3"/>
       <c r="J14" s="13"/>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="9"/>
-      <c r="B15" s="26"/>
+      <c r="B15" s="21"/>
       <c r="C15" s="10" t="s">
         <v>9</v>
       </c>
@@ -870,9 +851,8 @@
       <c r="I15" s="11"/>
       <c r="J15" s="14"/>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="2"/>
-      <c r="B16" s="27"/>
       <c r="E16" s="3"/>
       <c r="F16" s="13"/>
       <c r="G16" s="3"/>
@@ -880,11 +860,11 @@
       <c r="I16" s="3"/>
       <c r="J16" s="13"/>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B17" s="28"/>
+      <c r="B17" s="22"/>
       <c r="C17" s="15" t="s">
         <v>27</v>
       </c>
@@ -896,9 +876,9 @@
       <c r="I17" s="5"/>
       <c r="J17" s="12"/>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="7"/>
-      <c r="B18" s="25"/>
+      <c r="B18" s="18"/>
       <c r="C18" s="16" t="s">
         <v>11</v>
       </c>
@@ -909,9 +889,9 @@
       <c r="I18" s="3"/>
       <c r="J18" s="13"/>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="9"/>
-      <c r="B19" s="26"/>
+      <c r="B19" s="21"/>
       <c r="C19" s="17" t="s">
         <v>12</v>
       </c>
@@ -922,6 +902,36 @@
       <c r="H19" s="14"/>
       <c r="I19" s="11"/>
       <c r="J19" s="14"/>
+    </row>
+    <row r="44" spans="2:2" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B44" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="45" spans="2:2" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B45" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="46" spans="2:2" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B46" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="47" spans="2:2" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B47" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="48" spans="2:2" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B48" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="49" spans="2:2" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B49" t="s">
+        <v>20</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -931,7 +941,7 @@
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G6:G19 E6:E19 I6:I19" xr:uid="{98D6ACD6-3225-430E-B99E-5C33FDF86D90}">
-      <formula1>$T$4:$T$8</formula1>
+      <formula1>$B$44:$B$49</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>